<commit_message>
Auto build isw_v2-dist from GitHub Actions (增量编译) - 2026-02-14 06:23:21
</commit_message>
<xml_diff>
--- a/backend/apps/static/import_template/新增设备导入模板.xlsx
+++ b/backend/apps/static/import_template/新增设备导入模板.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26820" windowHeight="12975"/>
+    <workbookView windowWidth="27945" windowHeight="12975"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -47,19 +47,19 @@
     <t>设备类型Key</t>
   </si>
   <si>
-    <t>设备序列号</t>
+    <t>设备安裝位置</t>
   </si>
   <si>
-    <t>设备安裝位置</t>
+    <t>设备描述</t>
+  </si>
+  <si>
+    <t>设备序列号</t>
   </si>
   <si>
     <t>父设备Key</t>
   </si>
   <si>
     <t>子设备地址</t>
-  </si>
-  <si>
-    <t>设备描述</t>
   </si>
 </sst>
 </file>
@@ -1049,11 +1049,11 @@
   <cols>
     <col min="1" max="1" width="18.75" customWidth="1"/>
     <col min="2" max="2" width="22.875" customWidth="1"/>
-    <col min="3" max="3" width="16.5" customWidth="1"/>
-    <col min="4" max="4" width="16.625" customWidth="1"/>
-    <col min="5" max="5" width="17.375" customWidth="1"/>
-    <col min="6" max="6" width="17.75" customWidth="1"/>
-    <col min="7" max="7" width="65.75" customWidth="1"/>
+    <col min="3" max="3" width="23.5" customWidth="1"/>
+    <col min="4" max="4" width="35.25" customWidth="1"/>
+    <col min="5" max="5" width="16.625" customWidth="1"/>
+    <col min="6" max="6" width="17.375" customWidth="1"/>
+    <col min="7" max="7" width="14.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" spans="1:10">

</xml_diff>